<commit_message>
Add missing web address validation
</commit_message>
<xml_diff>
--- a/wwwroot/templates/CariTemplate.xlsx
+++ b/wwwroot/templates/CariTemplate.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MOD\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\EMutabakat\wwwroot\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C03ED3BD-EC37-445A-860F-3F94EDBBA246}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9D95F4B-286C-4191-917B-475252D1BB8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5685" yWindow="4485" windowWidth="16950" windowHeight="11115" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7485" yWindow="1380" windowWidth="16950" windowHeight="10950" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Worksheet" sheetId="1" r:id="rId1"/>
@@ -91,9 +91,6 @@
     <t>3456789012</t>
   </si>
   <si>
-    <t>www.abcgida.com</t>
-  </si>
-  <si>
     <t>Ahmet Yılmaz</t>
   </si>
   <si>
@@ -124,9 +121,6 @@
     <t>4567890123</t>
   </si>
   <si>
-    <t>www.maviyazilim.com</t>
-  </si>
-  <si>
     <t>Ayşe Demir</t>
   </si>
   <si>
@@ -157,9 +151,6 @@
     <t>5678901234</t>
   </si>
   <si>
-    <t>www.egemedikal.com</t>
-  </si>
-  <si>
     <t>Mehmet Kaya</t>
   </si>
   <si>
@@ -196,9 +187,6 @@
     <t>6789012345</t>
   </si>
   <si>
-    <t>www.ankalojistik.com</t>
-  </si>
-  <si>
     <t>Zeynep Çelik</t>
   </si>
   <si>
@@ -215,6 +203,18 @@
   </si>
   <si>
     <t>TL</t>
+  </si>
+  <si>
+    <t>https://abcgida.com</t>
+  </si>
+  <si>
+    <t>https://maviyazilim.com</t>
+  </si>
+  <si>
+    <t>https://egemedikal.com</t>
+  </si>
+  <si>
+    <t>https://ankalojistik.com</t>
   </si>
 </sst>
 </file>
@@ -254,12 +254,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -552,23 +555,23 @@
       <c r="I2" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="J2" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="K2" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="L2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="L2" s="1" t="s">
+      <c r="M2" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="M2" s="1" t="s">
+      <c r="N2" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="N2" s="2" t="s">
-        <v>27</v>
-      </c>
       <c r="O2" s="1" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="P2">
         <v>1</v>
@@ -582,43 +585,43 @@
         <v>2</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="E3" s="1" t="s">
         <v>29</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>30</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>19</v>
       </c>
       <c r="G3" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="H3" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="I3" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="J3" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="K3" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="J3" s="1" t="s">
+      <c r="L3" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="K3" s="1" t="s">
+      <c r="M3" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="L3" s="1" t="s">
+      <c r="N3" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="M3" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="N3" s="1" t="s">
-        <v>38</v>
-      </c>
       <c r="O3" s="1" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="P3">
         <v>1</v>
@@ -632,43 +635,43 @@
         <v>1</v>
       </c>
       <c r="C4" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="F4" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="G4" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="H4" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="I4" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="J4" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="K4" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="H4" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="I4" s="1" t="s">
+      <c r="L4" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J4" s="1" t="s">
+      <c r="M4" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="K4" s="1" t="s">
+      <c r="N4" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="L4" s="1" t="s">
+      <c r="O4" s="1" t="s">
         <v>47</v>
-      </c>
-      <c r="M4" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="N4" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="O4" s="1" t="s">
-        <v>50</v>
       </c>
       <c r="P4">
         <v>1</v>
@@ -682,49 +685,55 @@
         <v>2</v>
       </c>
       <c r="C5" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="F5" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="G5" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="H5" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="I5" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="J5" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="K5" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="H5" s="1" t="s">
+      <c r="L5" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="I5" s="1" t="s">
+      <c r="M5" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="J5" s="1" t="s">
+      <c r="N5" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="K5" s="1" t="s">
+      <c r="O5" s="1" t="s">
         <v>59</v>
-      </c>
-      <c r="L5" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="M5" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="N5" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="O5" s="1" t="s">
-        <v>63</v>
       </c>
       <c r="P5">
         <v>1</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="J2" r:id="rId1" xr:uid="{85A614E9-06B1-426D-9195-398702F2FF7D}"/>
+    <hyperlink ref="J3" r:id="rId2" xr:uid="{DFD0F7D7-800B-4948-8FA3-19FCA6FEBCED}"/>
+    <hyperlink ref="J4" r:id="rId3" xr:uid="{48E6E11E-AA42-4547-AD51-50A94EF1EC9D}"/>
+    <hyperlink ref="J5" r:id="rId4" xr:uid="{3B6D6488-D37C-490D-877B-FD4D00B3385D}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>